<commit_message>
PIES from flat conversion - XLSX upload
</commit_message>
<xml_diff>
--- a/PIES_7-1_flat_template_2020-05-13.xlsx
+++ b/PIES_7-1_flat_template_2020-05-13.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\APS36\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\APS36\Documents\NetBeansProjects\sandpim\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12435" tabRatio="809"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12435" tabRatio="809" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="Header" sheetId="2" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1354" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1356" uniqueCount="441">
   <si>
     <t>UP</t>
   </si>
@@ -1362,6 +1362,9 @@
   </si>
   <si>
     <t>Pleat Count</t>
+  </si>
+  <si>
+    <t>Component</t>
   </si>
 </sst>
 </file>
@@ -7480,9 +7483,22 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>440</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>